<commit_message>
fixed the python script for sttram write count analysis, still need to sort out the excel file formatting
</commit_message>
<xml_diff>
--- a/sttram_analysis_results.xlsx
+++ b/sttram_analysis_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/talhaahmed/Desktop/L3-Project/multi-retention-sttram-btb/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C42A4CD2-B8A2-EA4A-BBA9-EAA6E2138B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C69CB16-DFFA-7340-AE42-B9FDE35D01EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sttramBTB writes" sheetId="1" r:id="rId1"/>
@@ -20,39 +20,57 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="17">
+  <si>
+    <t>no_sttramBTB Stats</t>
+  </si>
+  <si>
+    <t>Partition ID</t>
+  </si>
+  <si>
+    <t>Offset Bits</t>
+  </si>
+  <si>
+    <t>Total Writes</t>
+  </si>
+  <si>
+    <t>% of Total</t>
+  </si>
+  <si>
+    <t>Return</t>
+  </si>
+  <si>
+    <t>&lt;= 4 bits</t>
+  </si>
+  <si>
+    <t>&lt;= 5 bits</t>
+  </si>
+  <si>
+    <t>&lt;= 7 bits</t>
+  </si>
+  <si>
+    <t>&lt;= 9 bits</t>
+  </si>
+  <si>
+    <t>&lt;= 11 bits</t>
+  </si>
+  <si>
+    <t>&lt;= 19 bits</t>
+  </si>
+  <si>
+    <t>&lt;= 25 bits</t>
+  </si>
+  <si>
+    <t>&gt; 25 bits</t>
+  </si>
   <si>
     <t>fdip_sttramBTB Stats</t>
   </si>
   <si>
-    <t>Way</t>
-  </si>
-  <si>
-    <t>Total Writes</t>
-  </si>
-  <si>
-    <t>Average Writes</t>
-  </si>
-  <si>
-    <t>Max Writes</t>
-  </si>
-  <si>
-    <t>no_sttramBTB Stats</t>
-  </si>
-  <si>
-    <t>Combined Averages</t>
-  </si>
-  <si>
-    <t>Combined Average Writes</t>
-  </si>
-  <si>
-    <t>Way Usage Summary</t>
-  </si>
-  <si>
-    <t>Count</t>
-  </si>
-  <si>
-    <t>Fraction</t>
+    <t>Combined Average Stats</t>
+  </si>
+  <si>
+    <t>Average Total Writes</t>
   </si>
 </sst>
 </file>
@@ -108,10 +126,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -415,128 +436,532 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
         <v>0</v>
       </c>
-      <c r="B3">
-        <v>398803966</v>
-      </c>
-      <c r="C3">
-        <v>1170.432967845697</v>
-      </c>
-      <c r="D3">
-        <v>1981550</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="C3" s="1">
+        <v>75527005</v>
+      </c>
+      <c r="D3" s="1">
+        <v>18.93840078870522</v>
+      </c>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
         <v>1</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1">
+        <v>64858623</v>
+      </c>
+      <c r="D4" s="1">
+        <v>16.263303396944369</v>
+      </c>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1">
+        <v>48242697</v>
+      </c>
+      <c r="D5" s="1">
+        <v>12.096859009755081</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="1">
+        <v>55789462</v>
+      </c>
+      <c r="D6" s="1">
+        <v>13.98921076166385</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>4</v>
+      </c>
       <c r="B7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="1">
+        <v>49444449</v>
+      </c>
+      <c r="D7" s="1">
+        <v>12.39819839193537</v>
+      </c>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1">
+        <v>30663668</v>
+      </c>
+      <c r="D8" s="1">
+        <v>7.6889164906750223</v>
+      </c>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="1">
+        <v>42716633</v>
+      </c>
+      <c r="D9" s="1">
+        <v>10.711198148238919</v>
+      </c>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="1">
+        <v>27413511</v>
+      </c>
+      <c r="D10" s="1">
+        <v>6.8739394385303516</v>
+      </c>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>8</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="1">
+        <v>4147451</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1.039973573551821</v>
+      </c>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D15" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8">
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
         <v>0</v>
       </c>
-      <c r="B8">
-        <v>398803499</v>
-      </c>
-      <c r="C8">
-        <v>1170.4315972670599</v>
-      </c>
-      <c r="D8">
-        <v>1981550</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="B16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="1">
+        <v>75527094</v>
+      </c>
+      <c r="D16" s="1">
+        <v>18.93840092854041</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
+        <v>1</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+      <c r="C17" s="1">
+        <v>64858698</v>
+      </c>
+      <c r="D17" s="1">
+        <v>16.263303158825661</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>2</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="1">
+        <v>48242748</v>
+      </c>
+      <c r="D18" s="1">
+        <v>12.09685763255424</v>
+      </c>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
+        <v>3</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="1">
+        <v>55789534</v>
+      </c>
+      <c r="D19" s="1">
+        <v>13.9892124342615</v>
+      </c>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>4</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="1">
+        <v>49444495</v>
+      </c>
+      <c r="D20" s="1">
+        <v>12.39819540811688</v>
+      </c>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>5</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="1">
+        <v>30663715</v>
+      </c>
+      <c r="D21" s="1">
+        <v>7.6889192721819626</v>
+      </c>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>6</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="1">
+        <v>42716667</v>
+      </c>
+      <c r="D22" s="1">
+        <v>10.7111941309029</v>
+      </c>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
+        <v>7</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="1">
+        <v>27413557</v>
+      </c>
+      <c r="D23" s="1">
+        <v>6.8739429236267924</v>
+      </c>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>8</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="1">
+        <v>4147458</v>
+      </c>
+      <c r="D24" s="1">
+        <v>1.039974110989659</v>
+      </c>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B28" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
+        <v>0</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29" s="1">
+        <v>75527049.5</v>
+      </c>
+      <c r="D29" s="1">
+        <v>18.93840085862286</v>
+      </c>
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
+        <v>1</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="1">
+        <v>64858660.5</v>
+      </c>
+      <c r="D30" s="1">
+        <v>16.26330327788494</v>
+      </c>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
+        <v>2</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>0</v>
-      </c>
-      <c r="B13">
-        <v>1170.4322825563791</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="C31" s="1">
+        <v>48242722.5</v>
+      </c>
+      <c r="D31" s="1">
+        <v>12.096858321154251</v>
+      </c>
+      <c r="E31" s="1"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
+        <v>3</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="1" t="s">
+      <c r="C32" s="1">
+        <v>55789498</v>
+      </c>
+      <c r="D32" s="1">
+        <v>13.98921159796317</v>
+      </c>
+      <c r="E32" s="1"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
+        <v>4</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C33" s="1">
+        <v>49444472</v>
+      </c>
+      <c r="D33" s="1">
+        <v>12.398196900025249</v>
+      </c>
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
+        <v>5</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18">
-        <v>0</v>
-      </c>
-      <c r="B18">
-        <v>797607465</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
+      <c r="C34" s="1">
+        <v>30663691.5</v>
+      </c>
+      <c r="D34" s="1">
+        <v>7.6889178814293064</v>
+      </c>
+      <c r="E34" s="1"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
+        <v>6</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C35" s="1">
+        <v>42716650</v>
+      </c>
+      <c r="D35" s="1">
+        <v>10.711196139569729</v>
+      </c>
+      <c r="E35" s="1"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
+        <v>7</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" s="1">
+        <v>27413534</v>
+      </c>
+      <c r="D36" s="1">
+        <v>6.8739411810795934</v>
+      </c>
+      <c r="E36" s="1"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
+        <v>8</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C37" s="1">
+        <v>4147454.5</v>
+      </c>
+      <c r="D37" s="1">
+        <v>1.0399738422708971</v>
+      </c>
+      <c r="E37" s="1"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>